<commit_message>
fix: empty rows before range and if not added to file
</commit_message>
<xml_diff>
--- a/example/generated.xlsx
+++ b/example/generated.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" tabRatio="204" windowHeight="8192" windowWidth="16384" xWindow="0" yWindow="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1" state="visible"/>
   </sheets>
   <definedNames/>
   <calcPr iterateCount="100" refMode="A1" iterateDelta="0.001"/>
@@ -16,19 +16,154 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>&lt;no value&gt;</t>
-  </si>
-  <si>
-    <t>{{ format_date .expire_date "2006-01-02" "02.01.2026" }}</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+  <si>
+    <t>Order #121231</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>MLDJIOND</t>
+  </si>
+  <si>
+    <t>5 998,37</t>
+  </si>
+  <si>
+    <t>8,06</t>
+  </si>
+  <si>
+    <t>13.02.2026</t>
+  </si>
+  <si>
+    <t>FGRVG</t>
+  </si>
+  <si>
+    <t>5 262,47</t>
+  </si>
+  <si>
+    <t>8,35</t>
+  </si>
+  <si>
+    <t>02.10.2025</t>
+  </si>
+  <si>
+    <t>XFLOHDVH</t>
+  </si>
+  <si>
+    <t>8 670,19</t>
+  </si>
+  <si>
+    <t>5,73</t>
+  </si>
+  <si>
+    <t>26.03.2025</t>
+  </si>
+  <si>
+    <t>TOZYZOA</t>
+  </si>
+  <si>
+    <t>171,87</t>
+  </si>
+  <si>
+    <t>5,23</t>
+  </si>
+  <si>
+    <t>25.01.2026</t>
+  </si>
+  <si>
+    <t>EORINLDH</t>
+  </si>
+  <si>
+    <t>1 464,13</t>
+  </si>
+  <si>
+    <t>7,62</t>
+  </si>
+  <si>
+    <t>16.05.2025</t>
+  </si>
+  <si>
+    <t>HKHARAS</t>
+  </si>
+  <si>
+    <t>4 893,98</t>
+  </si>
+  <si>
+    <t>0,50</t>
+  </si>
+  <si>
+    <t>20.07.2025</t>
+  </si>
+  <si>
+    <t>TUVQLU</t>
+  </si>
+  <si>
+    <t>4 831,42</t>
+  </si>
+  <si>
+    <t>2,21</t>
+  </si>
+  <si>
+    <t>19.09.2025</t>
+  </si>
+  <si>
+    <t>BGHPG</t>
+  </si>
+  <si>
+    <t>4 762,36</t>
+  </si>
+  <si>
+    <t>3,46</t>
+  </si>
+  <si>
+    <t>04.05.2025</t>
+  </si>
+  <si>
+    <t>PCBRAFC</t>
+  </si>
+  <si>
+    <t>5 380,33</t>
+  </si>
+  <si>
+    <t>3,44</t>
+  </si>
+  <si>
+    <t>09.09.2025</t>
+  </si>
+  <si>
+    <t>VQTMFICD</t>
+  </si>
+  <si>
+    <t>2 431,88</t>
+  </si>
+  <si>
+    <t>0,15</t>
+  </si>
+  <si>
+    <t>24.12.2025</t>
+  </si>
+  <si>
+    <t>Lucky customer</t>
+  </si>
+  <si>
+    <t>Test HyperLink</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Arial"/>
@@ -37,11 +172,32 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
+      <sz val="10"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <charset val="204"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
       <color rgb="FF000000"/>
+      <b/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <color rgb="FF0000FF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -74,18 +230,27 @@
       <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf applyAlignment="0" applyBorder="0" applyFont="0" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="0" numFmtId="0">
       <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0">
+      <alignment horizontal="center" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0">
+      <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="1" applyProtection="0" borderId="1" fillId="0" fontId="1" numFmtId="4" xfId="0">
-      <alignment horizontal="general" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
+      <alignment horizontal="center" indent="0" shrinkToFit="0" textRotation="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="0" applyNumberFormat="0" applyProtection="0" borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0">
+      <alignment horizontal="center" indent="0" shrinkToFit="0" textRotation="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -416,216 +581,197 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="12.85"/>
   <cols>
-    <col collapsed="false" hidden="false" max="2" min="2" style="0" width="12.52" customWidth="true"/>
-    <col collapsed="false" hidden="false" max="3" min="3" style="1" width="46.45" customWidth="true"/>
-    <col collapsed="false" hidden="false" max="4" min="4" style="1" width="28.22" customWidth="true"/>
-    <col collapsed="false" hidden="false" max="6" min="6" style="1" width="25.44" customWidth="true"/>
-    <col collapsed="false" hidden="false" max="7" min="7" style="1" width="15.69" customWidth="true"/>
+    <col collapsed="false" hidden="false" max="1" min="1" style="1" width="32.41" customWidth="true"/>
+    <col collapsed="false" hidden="false" max="2" min="2" style="1" width="32.69" customWidth="true"/>
+    <col collapsed="false" hidden="false" max="5" min="5" style="1" width="45.35" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="true">
+    <row r="1" ht="13.8" customHeight="true">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="2" t="s">
+    </row>
+    <row r="2" ht="13.8" customHeight="true">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" ht="14.25" customHeight="true">
-      <c r="B2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" ht="14.25" customHeight="true">
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="14.25" customHeight="true">
-      <c r="B4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="14.25" customHeight="true">
-      <c r="B5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="14.25" customHeight="true">
-      <c r="B6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" ht="14.25" customHeight="true">
-      <c r="B7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" ht="14.25" customHeight="true">
-      <c r="B8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" ht="14.25" customHeight="true">
-      <c r="B9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" ht="14.25" customHeight="true">
-      <c r="B10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" ht="12.8" customHeight="true">
+      <c r="B3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" ht="12.8" customHeight="true">
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" ht="12.8" customHeight="true">
+      <c r="B5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" ht="12.8" customHeight="true">
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="12.8" customHeight="true">
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" ht="12.8" customHeight="true">
+      <c r="B8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="12.8" customHeight="true">
+      <c r="B9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" ht="12.8" customHeight="true">
+      <c r="B10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" ht="12.8" customHeight="true">
+      <c r="B11" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" ht="12.8" customHeight="true">
+      <c r="B12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" ht="12.8" customHeight="true">
+      <c r="B14" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" ht="12.8" customHeight="true">
+      <c r="B17" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="B17:E23"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B17" display="Test HyperLink"/>
+  </hyperlinks>
 </worksheet>
 </file>
</xml_diff>